<commit_message>
Update documentation for interactive calculator
</commit_message>
<xml_diff>
--- a/materials/MedEd-HalluScore_Evaluation_Template_v0.2.xlsx
+++ b/materials/MedEd-HalluScore_Evaluation_Template_v0.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R03b4168935b44591"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluations" sheetId="2" r:id="R5fd56a933f904411"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rubric" sheetId="3" r:id="R93aeeae4f5734150"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Levels" sheetId="4" r:id="Ra95e9ef2912643e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R2067c387b04548cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluations" sheetId="2" r:id="R158505e0d0384b74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rubric" sheetId="3" r:id="R58967da687374695"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Levels" sheetId="4" r:id="Rbebf426978db4e25"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Strengthen rubric anchors and user guidance
</commit_message>
<xml_diff>
--- a/materials/MedEd-HalluScore_Evaluation_Template_v0.2.xlsx
+++ b/materials/MedEd-HalluScore_Evaluation_Template_v0.2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R2067c387b04548cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluations" sheetId="2" r:id="R158505e0d0384b74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rubric" sheetId="3" r:id="R58967da687374695"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Levels" sheetId="4" r:id="Rbebf426978db4e25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R131b62fa76a44531"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluations" sheetId="2" r:id="R6a57c4e316bc450e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rubric" sheetId="3" r:id="R03e2a8d1d46f451c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Levels" sheetId="4" r:id="R68c8e3eb716b4612"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1319,13 +1319,13 @@
         <x:v>Medical Factuality</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>No apparent factual error.</x:v>
+        <x:v>Accurate and current.</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Minor factual issue.</x:v>
+        <x:v>Minor imprecision.</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>Moderate error / Severe unsafe error.</x:v>
+        <x:v>Significant factual error / Critical dangerous error.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1361,13 +1361,13 @@
         <x:v>Clinical Reasoning Risk</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Appropriate reasoning.</x:v>
+        <x:v>Appropriate explicit reasoning.</x:v>
       </x:c>
       <x:c r="C5" t="str">
         <x:v>Mild oversimplification.</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>Incomplete or biased / Dangerous reasoning pattern.</x:v>
+        <x:v>Premature closure or bias / Dangerous heuristic.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1375,13 +1375,13 @@
         <x:v>Educational Safety</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Suitable after routine review.</x:v>
+        <x:v>Pedagogically appropriate.</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>Requires minor corrections.</x:v>
+        <x:v>Minor learner-level or clarity issue.</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>Requires substantial revision / Full rewrite.</x:v>
+        <x:v>Distorts learner priorities / Pedagogically unsafe.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1389,13 +1389,13 @@
         <x:v>Transparency and Verifiability</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Claims are clear and verifiable.</x:v>
+        <x:v>Clear and traceable claims.</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Some claims lack context.</x:v>
+        <x:v>Some context missing.</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>Many vague claims / Invented or nontraceable claims.</x:v>
+        <x:v>Hard to verify / Invented or falsely authoritative claim.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1562,7 +1562,7 @@
         <x:v>High Risk</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Do not use without substantial revision and re-review.</x:v>
+        <x:v>Multiple compromised dimensions; major revision and re-review required.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1573,7 +1573,7 @@
         <x:v>Critical Risk</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>Reject or fully rewrite before educational use.</x:v>
+        <x:v>Severe multi-dimensional risk; reject or fully rewrite before educational use.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>